<commit_message>
updates in user and case handling
</commit_message>
<xml_diff>
--- a/backend/data/users/radiology/user_1/rating_user_1.xlsx
+++ b/backend/data/users/radiology/user_1/rating_user_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,101 +427,6 @@
           <t>case_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>q1</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>q2</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>q3</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>q4</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>q5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>a2</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>a2</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>a5</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>a3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>a3</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>a2</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>a2</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>a4</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>a3</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>